<commit_message>
Initial push of AI Trust Index v1..1
</commit_message>
<xml_diff>
--- a/data/New Microsoft Excel Worksheet.xlsx
+++ b/data/New Microsoft Excel Worksheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D_DRIVE\Website_Projects\ai-trust-authority\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D_DRIVE\Website_Projects\ai-trust-authority\Auditai_git\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D9C7D7-E2A9-4F7D-945E-CF7BC7CDD11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A589322E-D5CC-42A7-B2F2-2233FE12DAC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1792,7 +1792,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1801,19 +1801,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1846,39 +1834,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1886,18 +1851,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2183,1029 +2144,1029 @@
   <dimension ref="A1:J32"/>
   <sheetFormatPr defaultColWidth="15.36328125" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="44.90625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="15.36328125" style="1"/>
+    <col min="1" max="1" width="36.7265625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="44.90625" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="15.36328125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="4">
         <v>46068</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="4">
         <v>46067</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="4">
         <v>46066</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="4">
         <v>46065</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="4">
         <v>46064</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>106</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="4">
         <v>46063</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="4">
         <v>46062</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="4">
         <v>46061</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="4">
         <v>46060</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="4">
         <v>46059</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="4">
         <v>46069</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="J12" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="4">
         <v>46069</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="I13" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="J13" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="4">
         <v>46070</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="J14" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="4">
         <v>46070</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="I15" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J15" s="9" t="s">
+      <c r="J15" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="4">
         <v>46071</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="I16" s="9" t="s">
+      <c r="I16" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="J16" s="9" t="s">
+      <c r="J16" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="4">
         <v>46071</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="I17" s="9" t="s">
+      <c r="I17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="J17" s="9" t="s">
+      <c r="J17" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="4">
         <v>46072</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="I18" s="9" t="s">
+      <c r="I18" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="J18" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="9" t="s">
+    <row r="19" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="4">
         <v>46072</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="J19" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="4">
         <v>46079</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="J20" s="9" t="s">
+      <c r="J20" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:10" s="12" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="13">
+      <c r="F21" s="4">
         <v>46074</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="2" t="s">
         <v>152</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="I21" s="14" t="s">
+      <c r="I21" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="J21" s="12" t="s">
+      <c r="J21" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="9" t="s">
+    <row r="22" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22" s="4">
         <v>46075</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="I22" s="9" t="s">
+      <c r="I22" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="J22" s="9" t="s">
+      <c r="J22" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
+    <row r="23" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="4">
         <v>46076</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="H23" s="11" t="s">
+      <c r="H23" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="I23" s="9" t="s">
+      <c r="I23" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="J23" s="9" t="s">
+      <c r="J23" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="9" t="s">
+    <row r="24" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="4">
         <v>46077</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="H24" s="11" t="s">
+      <c r="H24" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="I24" s="9" t="s">
+      <c r="I24" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="J24" s="9" t="s">
+      <c r="J24" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:10" s="9" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="9" t="s">
+    <row r="25" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F25" s="4">
         <v>46077</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="I25" s="9" t="s">
+      <c r="I25" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="J25" s="9" t="s">
+      <c r="J25" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:10" s="15" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="15" t="s">
+    <row r="26" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="E26" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F26" s="16">
+      <c r="F26" s="4">
         <v>46073</v>
       </c>
-      <c r="G26" s="15" t="s">
+      <c r="G26" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="I26" s="15" t="s">
+      <c r="I26" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="J26" s="15" t="s">
+      <c r="J26" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:10" s="15" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="15" t="s">
+    <row r="27" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E27" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="4">
         <v>46075</v>
       </c>
-      <c r="G27" s="15" t="s">
+      <c r="G27" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="I27" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="J27" s="15" t="s">
+      <c r="J27" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:10" s="5" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="5" t="s">
+    <row r="28" spans="1:10" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="7">
         <v>46078</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="G28" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="I28" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="J28" s="5" t="s">
+      <c r="J28" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:10" s="5" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="1:10" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="7">
         <v>46078</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="G29" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H29" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="I29" s="5" t="s">
+      <c r="I29" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="J29" s="5" t="s">
+      <c r="J29" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:10" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="30" spans="1:10" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="F30" s="18">
+      <c r="F30" s="7">
         <v>46076</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I30" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:10" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="31" spans="1:10" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="F31" s="18">
+      <c r="F31" s="7">
         <v>46074</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="H31" s="19" t="s">
+      <c r="H31" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:10" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="32" spans="1:10" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F32" s="18">
+      <c r="F32" s="7">
         <v>46073</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="H32" s="19" t="s">
+      <c r="H32" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="6" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>